<commit_message>
PROVA - alcune prove
</commit_message>
<xml_diff>
--- a/PS-VRP/Dati_input/Commesse_da_tagliare.xlsx
+++ b/PS-VRP/Dati_input/Commesse_da_tagliare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Frenc\Documents\GitHub\progettoIS\PS-VRP\Dati_input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76239B68-E5B6-4996-9FD4-0DB90BA00F75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0676DBF-7DB1-4897-8AFA-9871981BC5D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -11118,5 +11118,6 @@
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
PROVA - risolti problemi
</commit_message>
<xml_diff>
--- a/PS-VRP/Dati_input/Commesse_da_tagliare.xlsx
+++ b/PS-VRP/Dati_input/Commesse_da_tagliare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Frenc\Documents\GitHub\progettoIS\PS-VRP\Dati_input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0676DBF-7DB1-4897-8AFA-9871981BC5D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE6A9781-7E2C-4124-8DC6-0CA7F8E1EF4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10245" yWindow="3465" windowWidth="16665" windowHeight="11640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -490,7 +490,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -500,12 +500,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -534,7 +528,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -578,16 +572,6 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -1033,105 +1017,106 @@
       </c>
     </row>
     <row r="2" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A2" s="5">
+      <c r="A2" s="9">
         <v>254967</v>
       </c>
-      <c r="B2" s="6">
+      <c r="B2" s="10">
         <v>45981</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="10">
         <v>45996</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="9">
         <v>0</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2" s="9">
         <v>31250</v>
       </c>
-      <c r="G2" s="5">
+      <c r="G2" s="9">
         <v>1100</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="H2" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="I2" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="J2" s="5">
+      <c r="J2" s="9">
         <v>179</v>
       </c>
-      <c r="K2" s="5">
+      <c r="K2" s="9">
         <v>537</v>
       </c>
-      <c r="L2" s="7" t="s">
+      <c r="L2" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="M2" s="7" t="s">
+      <c r="M2" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="N2" s="7" t="s">
+      <c r="N2" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="O2" s="7" t="s">
+      <c r="O2" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="P2" s="7" t="s">
+      <c r="P2" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="Q2" s="7" t="s">
+      <c r="Q2" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="R2" s="7" t="s">
+      <c r="R2" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="S2" s="7" t="s">
+      <c r="S2" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="T2" s="7" t="s">
+      <c r="T2" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="U2" s="7" t="s">
+      <c r="U2" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="V2" s="7" t="s">
+      <c r="V2" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="W2" s="7" t="s">
+      <c r="W2" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="X2" s="7" t="s">
+      <c r="X2" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="Y2" s="7" t="s">
+      <c r="Y2" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="Z2" s="7" t="s">
+      <c r="Z2" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="AA2" s="7" t="s">
+      <c r="AA2" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="AB2" s="7" t="s">
+      <c r="AB2" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="AC2" s="7" t="s">
+      <c r="AC2" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="AD2" s="7" t="s">
+      <c r="AD2" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="AE2" s="7" t="s">
+      <c r="AE2" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="AF2" s="2">
+      <c r="AF2" s="9">
         <v>0</v>
       </c>
-      <c r="AG2" s="2">
+      <c r="AG2" s="9">
         <v>66</v>
       </c>
+      <c r="AH2" s="12"/>
     </row>
     <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
@@ -1737,100 +1722,100 @@
       </c>
     </row>
     <row r="9" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A9" s="2">
+      <c r="A9" s="9">
         <v>254671</v>
       </c>
-      <c r="B9" s="3">
+      <c r="B9" s="10">
         <v>45979</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="10">
         <v>45982</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="9">
         <v>0</v>
       </c>
-      <c r="F9" s="2">
+      <c r="F9" s="9">
         <v>16340</v>
       </c>
-      <c r="G9" s="2">
+      <c r="G9" s="9">
         <v>300</v>
       </c>
-      <c r="H9" s="4" t="s">
+      <c r="H9" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="I9" s="4" t="s">
+      <c r="I9" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="9">
         <v>110</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="9">
         <v>660</v>
       </c>
-      <c r="L9" s="4" t="s">
+      <c r="L9" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="M9" s="4" t="s">
+      <c r="M9" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="N9" s="4" t="s">
+      <c r="N9" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="O9" s="4" t="s">
+      <c r="O9" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="P9" s="4" t="s">
+      <c r="P9" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="Q9" s="4" t="s">
+      <c r="Q9" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="R9" s="4" t="s">
+      <c r="R9" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="S9" s="4" t="s">
+      <c r="S9" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="T9" s="4" t="s">
+      <c r="T9" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="U9" s="4" t="s">
+      <c r="U9" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="V9" s="4" t="s">
+      <c r="V9" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="W9" s="4" t="s">
+      <c r="W9" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="X9" s="4" t="s">
+      <c r="X9" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="Y9" s="4" t="s">
+      <c r="Y9" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="Z9" s="4" t="s">
+      <c r="Z9" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="AA9" s="4" t="s">
+      <c r="AA9" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="AB9" s="4" t="s">
+      <c r="AB9" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="AC9" s="4" t="s">
+      <c r="AC9" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="AD9" s="4" t="s">
+      <c r="AD9" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="AE9" s="4" t="s">
+      <c r="AE9" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="AF9" s="2">
+      <c r="AF9" s="9">
         <v>2</v>
       </c>
       <c r="AG9" s="2">
@@ -2634,95 +2619,95 @@
       </c>
     </row>
     <row r="18" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A18" s="13">
+      <c r="A18" s="9">
         <v>254428</v>
       </c>
-      <c r="B18" s="14">
+      <c r="B18" s="10">
         <v>45978</v>
       </c>
-      <c r="C18" s="15" t="s">
+      <c r="C18" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="D18" s="14">
+      <c r="D18" s="10">
         <v>45971</v>
       </c>
-      <c r="E18" s="13">
+      <c r="E18" s="9">
         <v>6</v>
       </c>
-      <c r="F18" s="13">
+      <c r="F18" s="9">
         <v>5797</v>
       </c>
-      <c r="G18" s="13">
+      <c r="G18" s="9">
         <v>300</v>
       </c>
-      <c r="H18" s="16"/>
-      <c r="I18" s="15" t="s">
+      <c r="H18" s="12"/>
+      <c r="I18" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="J18" s="13">
+      <c r="J18" s="9">
         <v>340</v>
       </c>
-      <c r="K18" s="13">
+      <c r="K18" s="9">
         <v>680</v>
       </c>
-      <c r="L18" s="15" t="s">
+      <c r="L18" s="11" t="s">
         <v>143</v>
       </c>
-      <c r="M18" s="15" t="s">
+      <c r="M18" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="N18" s="15" t="s">
+      <c r="N18" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="O18" s="15" t="s">
+      <c r="O18" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="P18" s="15" t="s">
+      <c r="P18" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="Q18" s="15" t="s">
+      <c r="Q18" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="R18" s="15" t="s">
+      <c r="R18" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="S18" s="15" t="s">
+      <c r="S18" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="T18" s="15" t="s">
+      <c r="T18" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="U18" s="15" t="s">
+      <c r="U18" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="V18" s="15" t="s">
+      <c r="V18" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="W18" s="15" t="s">
+      <c r="W18" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="X18" s="15" t="s">
+      <c r="X18" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="Y18" s="15" t="s">
+      <c r="Y18" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="Z18" s="15" t="s">
+      <c r="Z18" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="AA18" s="15" t="s">
+      <c r="AA18" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="AB18" s="15" t="s">
+      <c r="AB18" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="AC18" s="15" t="s">
+      <c r="AC18" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="AD18" s="15" t="s">
+      <c r="AD18" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="AE18" s="15" t="s">
+      <c r="AE18" s="11" t="s">
         <v>88</v>
       </c>
       <c r="AF18" s="2">
@@ -3036,93 +3021,93 @@
       </c>
     </row>
     <row r="22" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A22" s="13">
+      <c r="A22" s="9">
         <v>254173</v>
       </c>
-      <c r="B22" s="14">
+      <c r="B22" s="10">
         <v>45976</v>
       </c>
-      <c r="C22" s="15" t="s">
+      <c r="C22" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="D22" s="14">
+      <c r="D22" s="10">
         <v>45950</v>
       </c>
-      <c r="E22" s="13">
+      <c r="E22" s="9">
         <v>6</v>
       </c>
-      <c r="F22" s="13">
+      <c r="F22" s="9">
         <v>24311</v>
       </c>
-      <c r="G22" s="13">
+      <c r="G22" s="9">
         <v>1024</v>
       </c>
-      <c r="H22" s="16"/>
-      <c r="I22" s="15" t="s">
+      <c r="H22" s="12"/>
+      <c r="I22" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="J22" s="13">
+      <c r="J22" s="9">
         <v>800</v>
       </c>
-      <c r="K22" s="13">
+      <c r="K22" s="9">
         <v>800</v>
       </c>
-      <c r="L22" s="15" t="s">
+      <c r="L22" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="M22" s="16"/>
-      <c r="N22" s="15" t="s">
+      <c r="M22" s="12"/>
+      <c r="N22" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="O22" s="15" t="s">
+      <c r="O22" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="P22" s="15" t="s">
+      <c r="P22" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="Q22" s="15" t="s">
+      <c r="Q22" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="R22" s="15" t="s">
+      <c r="R22" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="S22" s="15" t="s">
+      <c r="S22" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="T22" s="15" t="s">
+      <c r="T22" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="U22" s="15" t="s">
+      <c r="U22" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="V22" s="15" t="s">
+      <c r="V22" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="W22" s="15" t="s">
+      <c r="W22" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="X22" s="15" t="s">
+      <c r="X22" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="Y22" s="15" t="s">
+      <c r="Y22" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="Z22" s="15" t="s">
+      <c r="Z22" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="AA22" s="15" t="s">
+      <c r="AA22" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="AB22" s="15" t="s">
+      <c r="AB22" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="AC22" s="15" t="s">
+      <c r="AC22" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="AD22" s="15" t="s">
+      <c r="AD22" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="AE22" s="15" t="s">
+      <c r="AE22" s="11" t="s">
         <v>82</v>
       </c>
       <c r="AF22" s="2">
@@ -8227,91 +8212,91 @@
       </c>
     </row>
     <row r="73" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A73" s="13">
+      <c r="A73" s="9">
         <v>252980</v>
       </c>
-      <c r="B73" s="14">
+      <c r="B73" s="10">
         <v>45972</v>
       </c>
-      <c r="C73" s="15" t="s">
+      <c r="C73" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="D73" s="14">
+      <c r="D73" s="10">
         <v>45908</v>
       </c>
-      <c r="E73" s="13">
+      <c r="E73" s="9">
         <v>6</v>
       </c>
-      <c r="F73" s="13">
+      <c r="F73" s="9">
         <v>2049</v>
       </c>
-      <c r="G73" s="13">
+      <c r="G73" s="9">
         <v>100</v>
       </c>
-      <c r="H73" s="15" t="s">
+      <c r="H73" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="I73" s="15" t="s">
+      <c r="I73" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="J73" s="16"/>
-      <c r="K73" s="13">
+      <c r="J73" s="12"/>
+      <c r="K73" s="9">
         <v>700</v>
       </c>
-      <c r="L73" s="16"/>
-      <c r="M73" s="16"/>
-      <c r="N73" s="15" t="s">
+      <c r="L73" s="12"/>
+      <c r="M73" s="12"/>
+      <c r="N73" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="O73" s="15" t="s">
+      <c r="O73" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="P73" s="15" t="s">
+      <c r="P73" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="Q73" s="15" t="s">
+      <c r="Q73" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="R73" s="15" t="s">
+      <c r="R73" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="S73" s="15" t="s">
+      <c r="S73" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="T73" s="15" t="s">
+      <c r="T73" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="U73" s="15" t="s">
+      <c r="U73" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="V73" s="15" t="s">
+      <c r="V73" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="W73" s="15" t="s">
+      <c r="W73" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="X73" s="15" t="s">
+      <c r="X73" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="Y73" s="15" t="s">
+      <c r="Y73" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="Z73" s="15" t="s">
+      <c r="Z73" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="AA73" s="15" t="s">
+      <c r="AA73" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="AB73" s="15" t="s">
+      <c r="AB73" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="AC73" s="15" t="s">
+      <c r="AC73" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="AD73" s="15" t="s">
+      <c r="AD73" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="AE73" s="15" t="s">
+      <c r="AE73" s="11" t="s">
         <v>82</v>
       </c>
       <c r="AF73" s="2">
@@ -8319,67 +8304,67 @@
       </c>
     </row>
     <row r="74" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A74" s="17">
+      <c r="A74" s="13">
         <v>254088</v>
       </c>
-      <c r="B74" s="18">
+      <c r="B74" s="14">
         <v>45972</v>
       </c>
-      <c r="C74" s="19" t="s">
+      <c r="C74" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="D74" s="18">
+      <c r="D74" s="14">
         <v>45950</v>
       </c>
-      <c r="E74" s="17">
+      <c r="E74" s="13">
         <v>1</v>
       </c>
-      <c r="F74" s="17">
+      <c r="F74" s="13">
         <v>51026</v>
       </c>
-      <c r="G74" s="17">
+      <c r="G74" s="13">
         <v>4000</v>
       </c>
-      <c r="H74" s="19" t="s">
+      <c r="H74" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="I74" s="19" t="s">
+      <c r="I74" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="J74" s="17">
+      <c r="J74" s="13">
         <v>270</v>
       </c>
-      <c r="K74" s="17">
+      <c r="K74" s="13">
         <v>810</v>
       </c>
-      <c r="L74" s="20"/>
-      <c r="M74" s="19" t="s">
+      <c r="L74" s="16"/>
+      <c r="M74" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="N74" s="19" t="s">
+      <c r="N74" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="O74" s="20"/>
-      <c r="P74" s="20"/>
-      <c r="Q74" s="20"/>
-      <c r="R74" s="20"/>
-      <c r="S74" s="20"/>
-      <c r="T74" s="20"/>
-      <c r="U74" s="20"/>
-      <c r="V74" s="20"/>
-      <c r="W74" s="20"/>
-      <c r="X74" s="20"/>
-      <c r="Y74" s="20"/>
-      <c r="Z74" s="20"/>
-      <c r="AA74" s="20"/>
-      <c r="AB74" s="20"/>
-      <c r="AC74" s="20"/>
-      <c r="AD74" s="20"/>
-      <c r="AE74" s="20"/>
-      <c r="AF74" s="17">
+      <c r="O74" s="16"/>
+      <c r="P74" s="16"/>
+      <c r="Q74" s="16"/>
+      <c r="R74" s="16"/>
+      <c r="S74" s="16"/>
+      <c r="T74" s="16"/>
+      <c r="U74" s="16"/>
+      <c r="V74" s="16"/>
+      <c r="W74" s="16"/>
+      <c r="X74" s="16"/>
+      <c r="Y74" s="16"/>
+      <c r="Z74" s="16"/>
+      <c r="AA74" s="16"/>
+      <c r="AB74" s="16"/>
+      <c r="AC74" s="16"/>
+      <c r="AD74" s="16"/>
+      <c r="AE74" s="16"/>
+      <c r="AF74" s="13">
         <v>2</v>
       </c>
-      <c r="AG74" s="17">
+      <c r="AG74" s="13">
         <v>378</v>
       </c>
     </row>
@@ -8674,102 +8659,105 @@
       </c>
     </row>
     <row r="78" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A78" s="2">
+      <c r="A78" s="9">
         <v>254609</v>
       </c>
-      <c r="B78" s="3">
+      <c r="B78" s="10">
         <v>45972</v>
       </c>
-      <c r="C78" s="4" t="s">
+      <c r="C78" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="D78" s="3">
+      <c r="D78" s="10">
         <v>45981</v>
       </c>
-      <c r="E78" s="2">
+      <c r="E78" s="9">
         <v>3</v>
       </c>
-      <c r="F78" s="2">
+      <c r="F78" s="9">
         <v>50000</v>
       </c>
-      <c r="G78" s="2">
+      <c r="G78" s="9">
         <v>2438</v>
       </c>
-      <c r="H78" s="4" t="s">
+      <c r="H78" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="I78" s="4" t="s">
+      <c r="I78" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="9">
         <v>400</v>
       </c>
-      <c r="K78" s="2">
+      <c r="K78" s="9">
         <v>750</v>
       </c>
-      <c r="L78" s="4" t="s">
+      <c r="L78" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="N78" s="4" t="s">
+      <c r="M78" s="12"/>
+      <c r="N78" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="O78" s="4" t="s">
+      <c r="O78" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="P78" s="4" t="s">
+      <c r="P78" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="Q78" s="4" t="s">
+      <c r="Q78" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="R78" s="4" t="s">
+      <c r="R78" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="S78" s="4" t="s">
+      <c r="S78" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="T78" s="4" t="s">
+      <c r="T78" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="U78" s="4" t="s">
+      <c r="U78" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="V78" s="4" t="s">
+      <c r="V78" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="W78" s="4" t="s">
+      <c r="W78" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="X78" s="4" t="s">
+      <c r="X78" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="Y78" s="4" t="s">
+      <c r="Y78" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="Z78" s="4" t="s">
+      <c r="Z78" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="AA78" s="4" t="s">
+      <c r="AA78" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="AB78" s="4" t="s">
+      <c r="AB78" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="AC78" s="4" t="s">
+      <c r="AC78" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="AD78" s="4" t="s">
+      <c r="AD78" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="AE78" s="4" t="s">
+      <c r="AE78" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="AF78" s="2">
+      <c r="AF78" s="9">
         <v>0</v>
       </c>
-      <c r="AG78" s="2">
+      <c r="AG78" s="9">
         <v>225</v>
       </c>
+      <c r="AH78" s="12"/>
+      <c r="AI78" s="12"/>
     </row>
     <row r="79" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A79" s="2">

</xml_diff>